<commit_message>
Update testing data for SPT processing
</commit_message>
<xml_diff>
--- a/spt/spt_processing_input.xlsx
+++ b/spt/spt_processing_input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eafit-my.sharepoint.com/personal/eamontoyaa_eafit_edu_co/Documents/EAMA/Dev/GitHub/EAFIT_slope_stability/notebooks/input_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eiaedu-my.sharepoint.com/personal/exneyder_montoya_eia_edu_co/Documents/EAMA/Dev/data4testing/spt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{C5008B80-3A1C-4689-B59D-AD5687BC6C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E21A449C-4E9C-40CB-9837-F7E1266BC79A}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{C5008B80-3A1C-4689-B59D-AD5687BC6C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7C44989-52C5-4734-AAC8-683A1CA80157}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7008F4F0-F30C-4941-AFE3-8359CC08712A}"/>
   </bookViews>
@@ -41,15 +41,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="13">
   <si>
     <t>Material</t>
   </si>
   <si>
     <t>Profundidad_(m)</t>
-  </si>
-  <si>
-    <t>Revestimiento_(m)</t>
   </si>
   <si>
     <t>Dep. Antrópico</t>
@@ -184,9 +181,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -224,7 +221,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -330,7 +327,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -472,7 +469,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -481,281 +478,238 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97243F2A-F833-4870-8595-53EB31C9E5F3}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C2" s="1">
         <v>0.3</v>
       </c>
       <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1">
         <v>1.3</v>
       </c>
       <c r="D3" s="1">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1">
-        <v>18</v>
-      </c>
-      <c r="F3" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1">
         <v>2.2999999999999998</v>
       </c>
       <c r="D4" s="1">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1">
         <v>0</v>
       </c>
-      <c r="E4" s="1">
-        <v>12</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="1">
         <v>3.3</v>
       </c>
       <c r="D5" s="1">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="1">
         <v>4.3</v>
       </c>
       <c r="D6" s="1">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E6" s="1">
-        <v>13</v>
-      </c>
-      <c r="F6" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="1">
         <v>5.3</v>
       </c>
       <c r="D7" s="1">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E7" s="1">
-        <v>11</v>
-      </c>
-      <c r="F7" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="1">
         <v>6.3</v>
       </c>
       <c r="D8" s="1">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E8" s="1">
-        <v>16</v>
-      </c>
-      <c r="F8" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" s="1">
         <v>7.3</v>
       </c>
       <c r="D9" s="1">
-        <v>2</v>
-      </c>
-      <c r="E9" s="1">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1">
         <v>8.3000000000000007</v>
       </c>
       <c r="D10" s="1">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E10" s="1">
-        <v>15</v>
-      </c>
-      <c r="F10" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1">
         <v>9.3000000000000007</v>
       </c>
       <c r="D11" s="1">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="E11" s="1">
-        <v>28</v>
-      </c>
-      <c r="F11" s="1">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12" s="1">
         <v>10.3</v>
       </c>
       <c r="D12" s="1">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E12" s="1">
-        <v>16</v>
-      </c>
-      <c r="F12" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C13" s="1">
         <v>11.3</v>
       </c>
       <c r="D13" s="1">
-        <v>2</v>
-      </c>
-      <c r="E13" s="1">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C14" s="1">
         <v>12.3</v>
       </c>
       <c r="D14" s="1">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E14" s="1">
-        <v>18</v>
-      </c>
-      <c r="F14" s="1">
         <v>49</v>
       </c>
     </row>
@@ -789,41 +743,47 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{a21f4c27-33e5-4cad-a1ff-6167bd9f9a45}" enabled="0" method="" siteId="{a21f4c27-33e5-4cad-a1ff-6167bd9f9a45}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>